<commit_message>
CD-222: Remove regular expressions from `givenName`, `familyName`, `affiliation`, `funding` and `library_prep_kit_version` fields
- The regex are specific/strict so they will void entries that should actually be okay. As a consequence, they are removed and users should enter free text in these fields.

- Applied the removal of the regex to the schemas - `singlecell_schema_main_v0.4.xlsx` and `reads_schema_main_v0.1.xlsx`

- Revised the error message for the `library_prep_kit_version` field
</commit_message>
<xml_diff>
--- a/single_cell/singlecell_schema_main_v0.4.xlsx
+++ b/single_cell/singlecell_schema_main_v0.4.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10810"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10927"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/providen/Documents/EI/Projects/COPO-schemas/single_cell/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8D5F6CE2-AB22-744E-B37D-5BC22BCE4D3C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{73F87B77-D407-844C-8ED8-2677A9C98583}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-680" yWindow="1840" windowWidth="26200" windowHeight="13060" activeTab="5" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
+    <workbookView xWindow="74460" yWindow="2080" windowWidth="26200" windowHeight="13060" xr2:uid="{7BD8D0E6-E1F4-E04F-9790-31602B31B6DB}"/>
   </bookViews>
   <sheets>
     <sheet name="data" sheetId="1" r:id="rId1"/>
@@ -81,7 +81,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3198" uniqueCount="1297">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3190" uniqueCount="1297">
   <si>
     <t>component_name</t>
   </si>
@@ -3992,9 +3992,6 @@
     <t>Expected a URL starting with 'http', 'https' or 'ftp'. For multiple URLs, separate them using the pipe symbol (|) with no spaces. e.g. https://reference-genome-example.com|https://example.org</t>
   </si>
   <si>
-    <t>Expected positive whole numbers or decimal numbers.</t>
-  </si>
-  <si>
     <t>Barcode sequence used on the i5 adapter during library preparation for identifying samples in multiplexed single-cell RNA-sequencing. The DNA barcode sequence (A, C, G, T), not a plate or well identifier should be specified.</t>
   </si>
   <si>
@@ -4104,6 +4101,9 @@
   </si>
   <si>
     <t>AND(LEN({column_letter}{row_start})=19,MID({column_letter}{row_start},5,1)="-",MID({column_letter}{row_start},10,1)="-",MID({column_letter}{row_start},15,1)="-",ISNUMBER(--LEFT({column_letter}{row_start},4)),ISNUMBER(--MID({column_letter}{row_start},6,4)),ISNUMBER(--MID({column_letter}{row_start},11,4)),ISNUMBER(--MID({column_letter}{row_start},16,3)),OR(ISNUMBER(--RIGHT({column_letter}{row_start},1)),RIGHT({column_letter}{row_start},1)="X"))</t>
+  </si>
+  <si>
+    <t>Expected a numeric version number.</t>
   </si>
 </sst>
 </file>
@@ -6374,12 +6374,8 @@
       <c r="J20" s="3" t="s">
         <v>116</v>
       </c>
-      <c r="K20" s="3" t="s">
-        <v>117</v>
-      </c>
-      <c r="L20" s="3" t="s">
-        <v>1205</v>
-      </c>
+      <c r="K20" s="3"/>
+      <c r="L20" s="3"/>
       <c r="M20" s="3" t="s">
         <v>24</v>
       </c>
@@ -6424,12 +6420,8 @@
       <c r="J21" s="3" t="s">
         <v>122</v>
       </c>
-      <c r="K21" s="3" t="s">
-        <v>123</v>
-      </c>
-      <c r="L21" s="3" t="s">
-        <v>1205</v>
-      </c>
+      <c r="K21" s="3"/>
+      <c r="L21" s="3"/>
       <c r="M21" s="3" t="s">
         <v>24</v>
       </c>
@@ -6524,12 +6516,8 @@
       <c r="J23" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="K23" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="L23" s="3" t="s">
-        <v>1205</v>
-      </c>
+      <c r="K23" s="3"/>
+      <c r="L23" s="3"/>
       <c r="M23" s="3" t="s">
         <v>24</v>
       </c>
@@ -6620,12 +6608,8 @@
       <c r="J25" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="K25" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="L25" s="3" t="s">
-        <v>1205</v>
-      </c>
+      <c r="K25" s="3"/>
+      <c r="L25" s="3"/>
       <c r="M25" s="3" t="s">
         <v>24</v>
       </c>
@@ -8187,13 +8171,13 @@
         <v>265</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>1262</v>
+        <v>1261</v>
       </c>
       <c r="F59" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I59" s="3" t="s">
-        <v>1263</v>
+        <v>1262</v>
       </c>
       <c r="J59" s="3" t="s">
         <v>256</v>
@@ -8576,7 +8560,7 @@
         <v>660</v>
       </c>
       <c r="L67" s="3" t="s">
-        <v>1259</v>
+        <v>1296</v>
       </c>
       <c r="M67" s="3" t="s">
         <v>24</v>
@@ -9156,7 +9140,7 @@
         <v>0</v>
       </c>
       <c r="I80" s="3" t="s">
-        <v>1260</v>
+        <v>1259</v>
       </c>
       <c r="J80" s="3" t="s">
         <v>336</v>
@@ -9200,7 +9184,7 @@
         <v>0</v>
       </c>
       <c r="I81" s="3" t="s">
-        <v>1261</v>
+        <v>1260</v>
       </c>
       <c r="J81" s="3" t="s">
         <v>339</v>
@@ -11188,16 +11172,16 @@
         <v>19</v>
       </c>
       <c r="C125" s="3" t="s">
+        <v>1263</v>
+      </c>
+      <c r="D125" s="3" t="s">
         <v>1264</v>
-      </c>
-      <c r="D125" s="3" t="s">
-        <v>1265</v>
       </c>
       <c r="F125" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I125" s="3" t="s">
-        <v>1266</v>
+        <v>1265</v>
       </c>
       <c r="J125" s="3">
         <v>12458</v>
@@ -11236,16 +11220,16 @@
         <v>19</v>
       </c>
       <c r="C126" s="3" t="s">
+        <v>1266</v>
+      </c>
+      <c r="D126" s="3" t="s">
         <v>1267</v>
-      </c>
-      <c r="D126" s="3" t="s">
-        <v>1268</v>
       </c>
       <c r="F126" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I126" s="3" t="s">
-        <v>1269</v>
+        <v>1268</v>
       </c>
       <c r="J126" s="3">
         <v>1842</v>
@@ -11284,19 +11268,19 @@
         <v>19</v>
       </c>
       <c r="C127" s="3" t="s">
+        <v>1269</v>
+      </c>
+      <c r="D127" s="3" t="s">
         <v>1270</v>
-      </c>
-      <c r="D127" s="3" t="s">
-        <v>1271</v>
       </c>
       <c r="F127" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I127" s="3" t="s">
+        <v>1271</v>
+      </c>
+      <c r="J127" s="3" t="s">
         <v>1272</v>
-      </c>
-      <c r="J127" s="3" t="s">
-        <v>1273</v>
       </c>
       <c r="K127" s="3"/>
       <c r="L127" s="3"/>
@@ -11328,16 +11312,16 @@
         <v>19</v>
       </c>
       <c r="C128" s="3" t="s">
+        <v>1273</v>
+      </c>
+      <c r="D128" s="3" t="s">
         <v>1274</v>
-      </c>
-      <c r="D128" s="3" t="s">
-        <v>1275</v>
       </c>
       <c r="F128" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I128" s="3" t="s">
-        <v>1276</v>
+        <v>1275</v>
       </c>
       <c r="J128" s="3">
         <v>8</v>
@@ -11376,19 +11360,19 @@
         <v>19</v>
       </c>
       <c r="C129" s="3" t="s">
+        <v>1276</v>
+      </c>
+      <c r="D129" s="3" t="s">
         <v>1277</v>
-      </c>
-      <c r="D129" s="3" t="s">
-        <v>1278</v>
       </c>
       <c r="F129" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I129" s="97" t="s">
+        <v>1278</v>
+      </c>
+      <c r="J129" s="3" t="s">
         <v>1279</v>
-      </c>
-      <c r="J129" s="3" t="s">
-        <v>1280</v>
       </c>
       <c r="K129" s="3"/>
       <c r="L129" s="3"/>
@@ -11420,25 +11404,25 @@
         <v>19</v>
       </c>
       <c r="C130" s="3" t="s">
+        <v>1280</v>
+      </c>
+      <c r="D130" s="3" t="s">
         <v>1281</v>
-      </c>
-      <c r="D130" s="3" t="s">
-        <v>1282</v>
       </c>
       <c r="F130" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I130" s="3" t="s">
-        <v>1283</v>
+        <v>1282</v>
       </c>
       <c r="J130" s="3">
         <v>0.62</v>
       </c>
       <c r="K130" s="3" t="s">
+        <v>1283</v>
+      </c>
+      <c r="L130" s="3" t="s">
         <v>1284</v>
-      </c>
-      <c r="L130" s="3" t="s">
-        <v>1285</v>
       </c>
       <c r="M130" s="3" t="s">
         <v>24</v>
@@ -11468,16 +11452,16 @@
         <v>19</v>
       </c>
       <c r="C131" s="3" t="s">
+        <v>1285</v>
+      </c>
+      <c r="D131" s="3" t="s">
         <v>1286</v>
-      </c>
-      <c r="D131" s="3" t="s">
-        <v>1287</v>
       </c>
       <c r="F131" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I131" s="97" t="s">
-        <v>1288</v>
+        <v>1287</v>
       </c>
       <c r="J131" s="3">
         <v>27</v>
@@ -11516,19 +11500,19 @@
         <v>19</v>
       </c>
       <c r="C132" s="3" t="s">
+        <v>1288</v>
+      </c>
+      <c r="D132" s="3" t="s">
         <v>1289</v>
-      </c>
-      <c r="D132" s="3" t="s">
-        <v>1290</v>
       </c>
       <c r="F132" s="1" t="b">
         <v>0</v>
       </c>
       <c r="I132" s="3" t="s">
+        <v>1290</v>
+      </c>
+      <c r="J132" s="3" t="s">
         <v>1291</v>
-      </c>
-      <c r="J132" s="3" t="s">
-        <v>1292</v>
       </c>
       <c r="K132" s="3"/>
       <c r="L132" s="3"/>
@@ -27456,7 +27440,7 @@
         <v>1257</v>
       </c>
       <c r="B63" s="48" t="s">
-        <v>1295</v>
+        <v>1294</v>
       </c>
       <c r="C63" s="49"/>
     </row>
@@ -27465,19 +27449,19 @@
         <v>1256</v>
       </c>
       <c r="B64" s="48" t="s">
-        <v>1296</v>
+        <v>1295</v>
       </c>
       <c r="C64" s="49"/>
     </row>
     <row r="65" spans="1:3" ht="34" x14ac:dyDescent="0.2">
       <c r="A65" s="48" t="s">
-        <v>1284</v>
+        <v>1283</v>
       </c>
       <c r="B65" s="48" t="s">
+        <v>1292</v>
+      </c>
+      <c r="C65" s="49" t="s">
         <v>1293</v>
-      </c>
-      <c r="C65" s="49" t="s">
-        <v>1294</v>
       </c>
     </row>
   </sheetData>

</xml_diff>